<commit_message>
sampling time is set to 40s based on Testo-350 specs
</commit_message>
<xml_diff>
--- a/MATLAB/Simulation/Data.xlsx
+++ b/MATLAB/Simulation/Data.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{934EA4D9-4E96-4AF1-98BF-65ABBF28749F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CC65685-DE4D-430E-959E-0635983DF61C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="27810" windowHeight="15480" tabRatio="725" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="27810" windowHeight="15480" tabRatio="725" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MonitoringScenarioParams" sheetId="7" r:id="rId1"/>
@@ -1443,7 +1443,7 @@
         <v>38</v>
       </c>
       <c r="B3" s="6">
-        <v>120</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>